<commit_message>
LESSON 16 - Finish creating test data - 09042025
</commit_message>
<xml_diff>
--- a/1. Database Design/Java23 QuyenPhan Database Design.xlsx
+++ b/1. Database Design/Java23 QuyenPhan Database Design.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28623"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\qphan\Desktop\bkit\course - webapp\java23\3. Database\1. Database Design\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD2DA501-580C-443E-9607-72818A602B0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2E68749-AECD-42AF-B262-33C7D66849E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14016" tabRatio="588" firstSheet="3" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" tabRatio="588" firstSheet="3" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="B1. Mô hình quan niệm" sheetId="1" r:id="rId1"/>
@@ -2493,6 +2493,9 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -2513,9 +2516,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2911,21 +2911,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A4:L24"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.6640625" customWidth="1"/>
-    <col min="2" max="2" width="16.5546875" customWidth="1"/>
-    <col min="3" max="3" width="12.6640625" customWidth="1"/>
-    <col min="4" max="4" width="20.6640625" customWidth="1"/>
-    <col min="5" max="8" width="16.88671875" customWidth="1"/>
-    <col min="9" max="9" width="12.6640625" customWidth="1"/>
-    <col min="10" max="10" width="18.6640625" customWidth="1"/>
+    <col min="1" max="1" width="14.7109375" customWidth="1"/>
+    <col min="2" max="2" width="16.5703125" customWidth="1"/>
+    <col min="3" max="3" width="12.7109375" customWidth="1"/>
+    <col min="4" max="4" width="20.7109375" customWidth="1"/>
+    <col min="5" max="8" width="16.85546875" customWidth="1"/>
+    <col min="9" max="9" width="12.7109375" customWidth="1"/>
+    <col min="10" max="10" width="18.7109375" customWidth="1"/>
     <col min="11" max="11" width="21" customWidth="1"/>
-    <col min="12" max="12" width="17.44140625" customWidth="1"/>
-    <col min="13" max="18" width="12.6640625" customWidth="1"/>
+    <col min="12" max="12" width="17.42578125" customWidth="1"/>
+    <col min="13" max="18" width="12.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="1" t="s">
         <v>0</v>
       </c>
@@ -2960,7 +2960,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="5" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="2" t="s">
         <v>1</v>
       </c>
@@ -2995,7 +2995,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="6" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="28" t="s">
         <v>118</v>
       </c>
@@ -3030,7 +3030,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="7" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>119</v>
       </c>
@@ -3060,7 +3060,7 @@
       <c r="K7" s="2"/>
       <c r="L7" s="2"/>
     </row>
-    <row r="8" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>120</v>
       </c>
@@ -3090,7 +3090,7 @@
       <c r="K8" s="2"/>
       <c r="L8" s="2"/>
     </row>
-    <row r="9" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="28" t="s">
         <v>90</v>
       </c>
@@ -3113,7 +3113,7 @@
       <c r="K9" s="2"/>
       <c r="L9" s="2"/>
     </row>
-    <row r="10" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="28" t="s">
         <v>117</v>
       </c>
@@ -3136,7 +3136,7 @@
       <c r="K10" s="2"/>
       <c r="L10" s="2"/>
     </row>
-    <row r="11" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="28" t="s">
         <v>116</v>
       </c>
@@ -3159,7 +3159,7 @@
       <c r="K11" s="2"/>
       <c r="L11" s="2"/>
     </row>
-    <row r="12" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="28" t="s">
         <v>115</v>
       </c>
@@ -3176,7 +3176,7 @@
       <c r="K12" s="2"/>
       <c r="L12" s="2"/>
     </row>
-    <row r="13" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B13" s="2" t="s">
         <v>14</v>
       </c>
@@ -3190,7 +3190,7 @@
       <c r="K13" s="2"/>
       <c r="L13" s="2"/>
     </row>
-    <row r="14" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
       <c r="D14" s="2"/>
@@ -3203,7 +3203,7 @@
       <c r="K14" s="2"/>
       <c r="L14" s="2"/>
     </row>
-    <row r="15" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
       <c r="D15" s="2"/>
@@ -3216,7 +3216,7 @@
       <c r="K15" s="2"/>
       <c r="L15" s="2"/>
     </row>
-    <row r="16" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
       <c r="D16" s="2"/>
@@ -3229,7 +3229,7 @@
       <c r="K16" s="2"/>
       <c r="L16" s="2"/>
     </row>
-    <row r="17" spans="2:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
       <c r="D17" s="2"/>
@@ -3242,7 +3242,7 @@
       <c r="K17" s="2"/>
       <c r="L17" s="2"/>
     </row>
-    <row r="18" spans="2:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>
       <c r="D18" s="2"/>
@@ -3255,7 +3255,7 @@
       <c r="K18" s="2"/>
       <c r="L18" s="2"/>
     </row>
-    <row r="19" spans="2:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
       <c r="D19" s="2"/>
@@ -3268,7 +3268,7 @@
       <c r="K19" s="2"/>
       <c r="L19" s="2"/>
     </row>
-    <row r="20" spans="2:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
       <c r="D20" s="2"/>
@@ -3281,12 +3281,12 @@
       <c r="K20" s="2"/>
       <c r="L20" s="2"/>
     </row>
-    <row r="22" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B22" s="14" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="24" spans="2:12" s="14" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="24" spans="2:12" s="14" customFormat="1" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -3297,27 +3297,27 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00967ACB-CFA1-460B-A734-E9F64BF353E8}">
   <dimension ref="A2:P58"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.6640625" customWidth="1"/>
+    <col min="1" max="1" width="14.7109375" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
-    <col min="3" max="3" width="14.33203125" customWidth="1"/>
-    <col min="4" max="5" width="20.6640625" customWidth="1"/>
-    <col min="6" max="9" width="16.88671875" customWidth="1"/>
-    <col min="10" max="10" width="12.6640625" customWidth="1"/>
-    <col min="11" max="13" width="18.6640625" customWidth="1"/>
+    <col min="3" max="3" width="14.28515625" customWidth="1"/>
+    <col min="4" max="5" width="20.7109375" customWidth="1"/>
+    <col min="6" max="9" width="16.85546875" customWidth="1"/>
+    <col min="10" max="10" width="12.7109375" customWidth="1"/>
+    <col min="11" max="13" width="18.7109375" customWidth="1"/>
     <col min="14" max="14" width="21" customWidth="1"/>
-    <col min="15" max="15" width="17.44140625" customWidth="1"/>
-    <col min="16" max="16" width="18.33203125" customWidth="1"/>
-    <col min="17" max="21" width="12.6640625" customWidth="1"/>
+    <col min="15" max="15" width="17.42578125" customWidth="1"/>
+    <col min="16" max="16" width="18.28515625" customWidth="1"/>
+    <col min="17" max="21" width="12.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="F2" s="14" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="4" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="1" t="s">
         <v>0</v>
       </c>
@@ -3361,7 +3361,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="5" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="30" t="s">
         <v>1</v>
       </c>
@@ -3405,7 +3405,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="6" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="28" t="s">
         <v>118</v>
       </c>
@@ -3449,7 +3449,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>119</v>
       </c>
@@ -3488,7 +3488,7 @@
       <c r="N7" s="2"/>
       <c r="O7" s="2"/>
     </row>
-    <row r="8" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>120</v>
       </c>
@@ -3521,7 +3521,7 @@
       <c r="N8" s="2"/>
       <c r="O8" s="2"/>
     </row>
-    <row r="9" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="28" t="s">
         <v>117</v>
       </c>
@@ -3547,7 +3547,7 @@
       <c r="N9" s="2"/>
       <c r="O9" s="2"/>
     </row>
-    <row r="10" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="28" t="s">
         <v>116</v>
       </c>
@@ -3571,7 +3571,7 @@
       <c r="N10" s="2"/>
       <c r="O10" s="2"/>
     </row>
-    <row r="11" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="28" t="s">
         <v>115</v>
       </c>
@@ -3595,7 +3595,7 @@
       <c r="N11" s="2"/>
       <c r="O11" s="2"/>
     </row>
-    <row r="12" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="2" t="s">
         <v>14</v>
       </c>
@@ -3615,7 +3615,7 @@
       <c r="N12" s="2"/>
       <c r="O12" s="2"/>
     </row>
-    <row r="13" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
       <c r="D13" s="2"/>
@@ -3630,7 +3630,7 @@
       <c r="N13" s="2"/>
       <c r="O13" s="2"/>
     </row>
-    <row r="14" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
       <c r="D14" s="2"/>
@@ -3646,7 +3646,7 @@
       <c r="N14" s="2"/>
       <c r="O14" s="2"/>
     </row>
-    <row r="15" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
       <c r="D15" s="2"/>
@@ -3662,7 +3662,7 @@
       <c r="N15" s="2"/>
       <c r="O15" s="2"/>
     </row>
-    <row r="16" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
       <c r="D16" s="2"/>
@@ -3678,7 +3678,7 @@
       <c r="N16" s="2"/>
       <c r="O16" s="2"/>
     </row>
-    <row r="17" spans="2:16" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
       <c r="D17" s="2"/>
@@ -3694,7 +3694,7 @@
       <c r="N17" s="2"/>
       <c r="O17" s="2"/>
     </row>
-    <row r="18" spans="2:16" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>
       <c r="D18" s="2"/>
@@ -3710,7 +3710,7 @@
       <c r="N18" s="2"/>
       <c r="O18" s="2"/>
     </row>
-    <row r="19" spans="2:16" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
       <c r="D19" s="2"/>
@@ -3726,7 +3726,7 @@
       <c r="N19" s="2"/>
       <c r="O19" s="2"/>
     </row>
-    <row r="20" spans="2:16" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
       <c r="D20" s="2"/>
@@ -3742,12 +3742,12 @@
       <c r="N20" s="2"/>
       <c r="O20" s="2"/>
     </row>
-    <row r="22" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B22" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="23" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B23" t="s">
         <v>65</v>
       </c>
@@ -3761,7 +3761,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="24" spans="2:16" s="14" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:16" s="14" customFormat="1" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B24"/>
       <c r="C24" t="s">
         <v>66</v>
@@ -3787,7 +3787,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="25" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B25" s="8" t="s">
         <v>67</v>
       </c>
@@ -3816,7 +3816,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="26" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B26" s="8" t="s">
         <v>68</v>
       </c>
@@ -3843,7 +3843,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="27" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:16" x14ac:dyDescent="0.25">
       <c r="C27" t="s">
         <v>69</v>
       </c>
@@ -3867,7 +3867,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="28" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:16" x14ac:dyDescent="0.25">
       <c r="H28" s="23" t="s">
         <v>139</v>
       </c>
@@ -3884,7 +3884,7 @@
       <c r="O28" s="23"/>
       <c r="P28" s="23"/>
     </row>
-    <row r="29" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:16" x14ac:dyDescent="0.25">
       <c r="H29" s="23" t="s">
         <v>139</v>
       </c>
@@ -3901,7 +3901,7 @@
       <c r="O29" s="23"/>
       <c r="P29" s="23"/>
     </row>
-    <row r="30" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:16" x14ac:dyDescent="0.25">
       <c r="G30" s="31" t="s">
         <v>141</v>
       </c>
@@ -3921,14 +3921,14 @@
       <c r="O30" s="23"/>
       <c r="P30" s="23"/>
     </row>
-    <row r="31" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:16" x14ac:dyDescent="0.25">
       <c r="N31" s="23" t="s">
         <v>101</v>
       </c>
       <c r="O31" s="23"/>
       <c r="P31" s="23"/>
     </row>
-    <row r="32" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:16" x14ac:dyDescent="0.25">
       <c r="N32" s="4" t="s">
         <v>102</v>
       </c>
@@ -3936,7 +3936,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="33" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:15" x14ac:dyDescent="0.25">
       <c r="N33" s="4">
         <v>1</v>
       </c>
@@ -3944,7 +3944,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="34" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:15" x14ac:dyDescent="0.25">
       <c r="H34" t="s">
         <v>0</v>
       </c>
@@ -3955,7 +3955,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="35" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:15" x14ac:dyDescent="0.25">
       <c r="H35" s="28" t="s">
         <v>1</v>
       </c>
@@ -3972,7 +3972,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="36" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:15" x14ac:dyDescent="0.25">
       <c r="H36" s="23" t="s">
         <v>132</v>
       </c>
@@ -3989,7 +3989,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="37" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:15" x14ac:dyDescent="0.25">
       <c r="H37" s="23" t="s">
         <v>133</v>
       </c>
@@ -4000,7 +4000,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="38" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:15" x14ac:dyDescent="0.25">
       <c r="H38" s="23" t="s">
         <v>134</v>
       </c>
@@ -4014,7 +4014,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="39" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B39" s="23"/>
       <c r="C39" s="23"/>
       <c r="D39" s="23"/>
@@ -4026,7 +4026,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="40" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B40" s="23"/>
       <c r="C40" s="23"/>
       <c r="D40" s="23"/>
@@ -4038,7 +4038,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="41" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="41" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B41" s="23"/>
       <c r="C41" s="23"/>
       <c r="D41" s="23"/>
@@ -4050,7 +4050,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="42" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="42" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B42" s="23"/>
       <c r="C42" s="23"/>
       <c r="D42" s="23"/>
@@ -4062,7 +4062,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="43" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="43" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B43" s="1" t="s">
         <v>160</v>
       </c>
@@ -4076,7 +4076,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="44" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="44" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B44" s="2" t="s">
         <v>104</v>
       </c>
@@ -4097,7 +4097,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="45" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="45" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B45" s="23" t="s">
         <v>159</v>
       </c>
@@ -4118,7 +4118,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="46" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="46" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B46" s="23" t="s">
         <v>159</v>
       </c>
@@ -4139,7 +4139,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="47" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="47" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B47" s="23" t="s">
         <v>159</v>
       </c>
@@ -4157,7 +4157,7 @@
       </c>
       <c r="G47" s="23"/>
     </row>
-    <row r="48" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="48" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B48" s="23"/>
       <c r="C48" s="23"/>
       <c r="D48" s="23"/>
@@ -4166,7 +4166,7 @@
       <c r="G48" s="23"/>
       <c r="H48" s="23"/>
     </row>
-    <row r="49" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="49" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B49" s="23"/>
       <c r="C49" s="23"/>
       <c r="D49" s="23"/>
@@ -4175,7 +4175,7 @@
       <c r="G49" s="23"/>
       <c r="H49" s="23"/>
     </row>
-    <row r="50" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="50" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B50" s="23" t="s">
         <v>127</v>
       </c>
@@ -4186,7 +4186,7 @@
       <c r="G50" s="23"/>
       <c r="H50" s="23"/>
     </row>
-    <row r="51" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="51" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B51" s="2" t="s">
         <v>104</v>
       </c>
@@ -4201,7 +4201,7 @@
       <c r="G51" s="23"/>
       <c r="H51" s="23"/>
     </row>
-    <row r="52" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="52" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B52" s="23" t="s">
         <v>159</v>
       </c>
@@ -4216,7 +4216,7 @@
       <c r="G52" s="23"/>
       <c r="H52" s="23"/>
     </row>
-    <row r="53" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="53" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B53" s="23" t="s">
         <v>161</v>
       </c>
@@ -4231,7 +4231,7 @@
       <c r="G53" s="23"/>
       <c r="H53" s="23"/>
     </row>
-    <row r="54" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="54" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B54" s="23" t="s">
         <v>162</v>
       </c>
@@ -4246,7 +4246,7 @@
       <c r="G54" s="23"/>
       <c r="H54" s="23"/>
     </row>
-    <row r="55" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="55" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B55" s="23"/>
       <c r="C55" s="23"/>
       <c r="D55" s="23"/>
@@ -4255,7 +4255,7 @@
       <c r="G55" s="23"/>
       <c r="H55" s="23"/>
     </row>
-    <row r="56" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="56" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B56" s="23"/>
       <c r="C56" s="23"/>
       <c r="D56" s="23"/>
@@ -4264,7 +4264,7 @@
       <c r="G56" s="23"/>
       <c r="H56" s="23"/>
     </row>
-    <row r="57" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="57" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B57" s="23"/>
       <c r="C57" s="23"/>
       <c r="D57" s="23"/>
@@ -4273,7 +4273,7 @@
       <c r="G57" s="23"/>
       <c r="H57" s="23"/>
     </row>
-    <row r="58" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="58" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B58" s="23"/>
       <c r="C58" s="23"/>
       <c r="D58" s="23"/>
@@ -4292,16 +4292,16 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A2:U43"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="4" max="4" width="10" customWidth="1"/>
-    <col min="8" max="8" width="13.6640625" customWidth="1"/>
-    <col min="9" max="9" width="10.44140625" customWidth="1"/>
-    <col min="15" max="15" width="12.5546875" customWidth="1"/>
-    <col min="16" max="16" width="11.88671875" customWidth="1"/>
+    <col min="8" max="8" width="13.7109375" customWidth="1"/>
+    <col min="9" max="9" width="10.42578125" customWidth="1"/>
+    <col min="15" max="15" width="12.5703125" customWidth="1"/>
+    <col min="16" max="16" width="11.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
         <v>76</v>
       </c>
@@ -4314,7 +4314,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>1</v>
       </c>
@@ -4322,7 +4322,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2</v>
       </c>
@@ -4331,10 +4331,10 @@
       </c>
       <c r="P4" s="25"/>
     </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:21" x14ac:dyDescent="0.25">
       <c r="N5" s="25"/>
     </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B7" s="9" t="s">
         <v>38</v>
       </c>
@@ -4346,7 +4346,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:21" x14ac:dyDescent="0.25">
       <c r="D8" s="4"/>
       <c r="P8" s="17" t="s">
         <v>54</v>
@@ -4355,7 +4355,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B9" s="5" t="s">
         <v>23</v>
       </c>
@@ -4396,7 +4396,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B10" s="3" t="s">
         <v>40</v>
       </c>
@@ -4437,7 +4437,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="11" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B11" s="3" t="s">
         <v>58</v>
       </c>
@@ -4472,7 +4472,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="12" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B12" s="3" t="s">
         <v>41</v>
       </c>
@@ -4507,7 +4507,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="13" spans="1:21" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:21" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B13" s="3" t="s">
         <v>52</v>
       </c>
@@ -4523,14 +4523,14 @@
       <c r="Q13" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="R13" s="62" t="s">
+      <c r="R13" s="63" t="s">
         <v>63</v>
       </c>
-      <c r="S13" s="62"/>
-      <c r="T13" s="62"/>
-      <c r="U13" s="62"/>
-    </row>
-    <row r="14" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="S13" s="63"/>
+      <c r="T13" s="63"/>
+      <c r="U13" s="63"/>
+    </row>
+    <row r="14" spans="1:21" x14ac:dyDescent="0.25">
       <c r="D14" s="4"/>
       <c r="O14" s="12" t="s">
         <v>38</v>
@@ -4541,20 +4541,20 @@
       <c r="Q14" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="R14" s="62"/>
-      <c r="S14" s="62"/>
-      <c r="T14" s="62"/>
-      <c r="U14" s="62"/>
-    </row>
-    <row r="15" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="R14" s="63"/>
+      <c r="S14" s="63"/>
+      <c r="T14" s="63"/>
+      <c r="U14" s="63"/>
+    </row>
+    <row r="15" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B15" s="4" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="16" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:21" x14ac:dyDescent="0.25">
       <c r="J16" s="25"/>
     </row>
-    <row r="17" spans="2:20" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B17" s="10" t="s">
         <v>32</v>
       </c>
@@ -4574,7 +4574,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="18" spans="2:20" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:20" x14ac:dyDescent="0.25">
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
       <c r="I18" s="4"/>
@@ -4585,7 +4585,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="19" spans="2:20" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B19" s="5" t="s">
         <v>33</v>
       </c>
@@ -4614,7 +4614,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="20" spans="2:20" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B20" s="11">
         <v>1</v>
       </c>
@@ -4637,7 +4637,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="21" spans="2:20" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B21" s="3" t="s">
         <v>49</v>
       </c>
@@ -4669,7 +4669,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="22" spans="2:20" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B22" s="3">
         <v>3</v>
       </c>
@@ -4696,7 +4696,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="23" spans="2:20" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:20" x14ac:dyDescent="0.25">
       <c r="G23" s="4">
         <v>4</v>
       </c>
@@ -4713,7 +4713,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="24" spans="2:20" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:20" x14ac:dyDescent="0.25">
       <c r="G24" s="4">
         <v>5</v>
       </c>
@@ -4727,7 +4727,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="25" spans="2:20" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:20" x14ac:dyDescent="0.25">
       <c r="G25" s="4">
         <v>6</v>
       </c>
@@ -4741,7 +4741,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="26" spans="2:20" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:20" x14ac:dyDescent="0.25">
       <c r="G26" s="4">
         <v>7</v>
       </c>
@@ -4758,7 +4758,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="27" spans="2:20" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:20" x14ac:dyDescent="0.25">
       <c r="N27" s="25" t="s">
         <v>1</v>
       </c>
@@ -4766,7 +4766,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="28" spans="2:20" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B28" t="s">
         <v>64</v>
       </c>
@@ -4777,7 +4777,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="29" spans="2:20" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B29" t="s">
         <v>65</v>
       </c>
@@ -4788,7 +4788,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="30" spans="2:20" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:20" x14ac:dyDescent="0.25">
       <c r="C30" t="s">
         <v>66</v>
       </c>
@@ -4799,7 +4799,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="31" spans="2:20" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B31" s="8" t="s">
         <v>67</v>
       </c>
@@ -4814,7 +4814,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="32" spans="2:20" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B32" s="8" t="s">
         <v>68</v>
       </c>
@@ -4832,7 +4832,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="33" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:15" x14ac:dyDescent="0.25">
       <c r="C33" t="s">
         <v>69</v>
       </c>
@@ -4843,7 +4843,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="34" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:15" x14ac:dyDescent="0.25">
       <c r="N34">
         <v>3</v>
       </c>
@@ -4851,7 +4851,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="35" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B35" t="s">
         <v>169</v>
       </c>
@@ -4863,7 +4863,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="36" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B36" t="s">
         <v>170</v>
       </c>
@@ -4871,31 +4871,31 @@
       <c r="I36" s="23"/>
       <c r="J36" s="23"/>
     </row>
-    <row r="37" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:15" x14ac:dyDescent="0.25">
       <c r="I37" s="23"/>
       <c r="J37" s="23"/>
     </row>
-    <row r="38" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:15" x14ac:dyDescent="0.25">
       <c r="I38" s="23"/>
       <c r="J38" s="23"/>
     </row>
-    <row r="39" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:15" x14ac:dyDescent="0.25">
       <c r="I39" s="23"/>
       <c r="J39" s="23"/>
     </row>
-    <row r="40" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:15" x14ac:dyDescent="0.25">
       <c r="I40" s="23"/>
       <c r="J40" s="23"/>
     </row>
-    <row r="41" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="41" spans="2:15" x14ac:dyDescent="0.25">
       <c r="I41" s="23"/>
       <c r="J41" s="23"/>
     </row>
-    <row r="42" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="42" spans="2:15" x14ac:dyDescent="0.25">
       <c r="I42" s="26"/>
       <c r="J42" s="26"/>
     </row>
-    <row r="43" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="43" spans="2:15" x14ac:dyDescent="0.25">
       <c r="I43" s="23"/>
       <c r="J43" s="23"/>
     </row>
@@ -4911,27 +4911,27 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7AD2C7DF-5616-418E-B427-D50946AF144B}">
   <dimension ref="A2:Q58"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.6640625" customWidth="1"/>
+    <col min="1" max="1" width="14.7109375" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
-    <col min="3" max="3" width="14.33203125" customWidth="1"/>
-    <col min="4" max="5" width="20.6640625" customWidth="1"/>
-    <col min="6" max="9" width="16.88671875" customWidth="1"/>
-    <col min="10" max="10" width="12.6640625" customWidth="1"/>
-    <col min="11" max="13" width="18.6640625" customWidth="1"/>
+    <col min="3" max="3" width="14.28515625" customWidth="1"/>
+    <col min="4" max="5" width="20.7109375" customWidth="1"/>
+    <col min="6" max="9" width="16.85546875" customWidth="1"/>
+    <col min="10" max="10" width="12.7109375" customWidth="1"/>
+    <col min="11" max="13" width="18.7109375" customWidth="1"/>
     <col min="14" max="14" width="21" customWidth="1"/>
-    <col min="15" max="15" width="17.44140625" customWidth="1"/>
-    <col min="16" max="16" width="18.33203125" customWidth="1"/>
-    <col min="17" max="21" width="12.6640625" customWidth="1"/>
+    <col min="15" max="15" width="17.42578125" customWidth="1"/>
+    <col min="16" max="16" width="18.28515625" customWidth="1"/>
+    <col min="17" max="21" width="12.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="F2" s="14" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="3" spans="1:15" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:15" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B3" s="4" t="s">
         <v>141</v>
       </c>
@@ -4972,7 +4972,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="4" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="1" t="s">
         <v>0</v>
       </c>
@@ -5016,7 +5016,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="5" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="30" t="s">
         <v>1</v>
       </c>
@@ -5060,7 +5060,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="6" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="28" t="s">
         <v>118</v>
       </c>
@@ -5104,7 +5104,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>119</v>
       </c>
@@ -5143,7 +5143,7 @@
       <c r="N7" s="2"/>
       <c r="O7" s="2"/>
     </row>
-    <row r="8" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>120</v>
       </c>
@@ -5176,7 +5176,7 @@
       <c r="N8" s="2"/>
       <c r="O8" s="2"/>
     </row>
-    <row r="9" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="28" t="s">
         <v>117</v>
       </c>
@@ -5202,7 +5202,7 @@
       <c r="N9" s="2"/>
       <c r="O9" s="2"/>
     </row>
-    <row r="10" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="28" t="s">
         <v>116</v>
       </c>
@@ -5226,7 +5226,7 @@
       <c r="N10" s="2"/>
       <c r="O10" s="2"/>
     </row>
-    <row r="11" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="28" t="s">
         <v>115</v>
       </c>
@@ -5250,7 +5250,7 @@
       <c r="N11" s="2"/>
       <c r="O11" s="2"/>
     </row>
-    <row r="12" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="2" t="s">
         <v>14</v>
       </c>
@@ -5270,7 +5270,7 @@
       <c r="N12" s="2"/>
       <c r="O12" s="2"/>
     </row>
-    <row r="13" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
       <c r="D13" s="2"/>
@@ -5285,7 +5285,7 @@
       <c r="N13" s="2"/>
       <c r="O13" s="2"/>
     </row>
-    <row r="14" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
       <c r="D14" s="2"/>
@@ -5301,7 +5301,7 @@
       <c r="N14" s="2"/>
       <c r="O14" s="2"/>
     </row>
-    <row r="15" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
       <c r="D15" s="2"/>
@@ -5317,7 +5317,7 @@
       <c r="N15" s="2"/>
       <c r="O15" s="2"/>
     </row>
-    <row r="16" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
       <c r="D16" s="2"/>
@@ -5333,7 +5333,7 @@
       <c r="N16" s="2"/>
       <c r="O16" s="2"/>
     </row>
-    <row r="17" spans="2:17" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:17" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
       <c r="D17" s="2"/>
@@ -5349,7 +5349,7 @@
       <c r="N17" s="2"/>
       <c r="O17" s="2"/>
     </row>
-    <row r="18" spans="2:17" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:17" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>
       <c r="D18" s="2"/>
@@ -5365,7 +5365,7 @@
       <c r="N18" s="2"/>
       <c r="O18" s="2"/>
     </row>
-    <row r="19" spans="2:17" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:17" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
       <c r="D19" s="2"/>
@@ -5381,7 +5381,7 @@
       <c r="N19" s="2"/>
       <c r="O19" s="2"/>
     </row>
-    <row r="20" spans="2:17" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:17" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
       <c r="D20" s="2"/>
@@ -5397,12 +5397,12 @@
       <c r="N20" s="2"/>
       <c r="O20" s="2"/>
     </row>
-    <row r="23" spans="2:17" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:17" x14ac:dyDescent="0.25">
       <c r="C23" s="32" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="24" spans="2:17" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:17" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B24"/>
       <c r="C24" s="16" t="s">
         <v>172</v>
@@ -5421,17 +5421,17 @@
       <c r="P24"/>
       <c r="Q24"/>
     </row>
-    <row r="25" spans="2:17" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:17" x14ac:dyDescent="0.25">
       <c r="C25" s="16" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="27" spans="2:17" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:17" x14ac:dyDescent="0.25">
       <c r="C27" s="32" t="s">
         <v>174</v>
       </c>
     </row>
-    <row r="28" spans="2:17" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:17" x14ac:dyDescent="0.25">
       <c r="C28" s="16" t="s">
         <v>175</v>
       </c>
@@ -5441,7 +5441,7 @@
       <c r="O28" s="23"/>
       <c r="P28" s="23"/>
     </row>
-    <row r="29" spans="2:17" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:17" x14ac:dyDescent="0.25">
       <c r="C29" s="16" t="s">
         <v>176</v>
       </c>
@@ -5451,47 +5451,47 @@
       <c r="O29" s="23"/>
       <c r="P29" s="23"/>
     </row>
-    <row r="30" spans="2:17" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:17" x14ac:dyDescent="0.25">
       <c r="L30" s="23"/>
       <c r="M30" s="23"/>
       <c r="N30" s="23"/>
       <c r="O30" s="23"/>
       <c r="P30" s="23"/>
     </row>
-    <row r="31" spans="2:17" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:17" x14ac:dyDescent="0.25">
       <c r="C31" s="32" t="s">
         <v>177</v>
       </c>
     </row>
-    <row r="32" spans="2:17" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:17" x14ac:dyDescent="0.25">
       <c r="C32" s="16" t="s">
         <v>178</v>
       </c>
     </row>
-    <row r="33" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:8" x14ac:dyDescent="0.25">
       <c r="C33" s="16" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="35" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:8" x14ac:dyDescent="0.25">
       <c r="C35" s="32" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="36" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:8" x14ac:dyDescent="0.25">
       <c r="C36" s="16" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="37" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:8" x14ac:dyDescent="0.25">
       <c r="C37" s="16"/>
     </row>
-    <row r="38" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:8" x14ac:dyDescent="0.25">
       <c r="C38" s="16" t="s">
         <v>182</v>
       </c>
     </row>
-    <row r="39" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B39" s="23"/>
       <c r="C39" s="33" t="s">
         <v>183</v>
@@ -5502,23 +5502,23 @@
       <c r="G39" s="23"/>
       <c r="H39" s="23"/>
     </row>
-    <row r="40" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:8" x14ac:dyDescent="0.25">
       <c r="G40" s="23"/>
       <c r="H40" s="23"/>
     </row>
-    <row r="41" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="41" spans="2:8" x14ac:dyDescent="0.25">
       <c r="G41" s="23"/>
       <c r="H41" s="23"/>
     </row>
-    <row r="42" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="42" spans="2:8" x14ac:dyDescent="0.25">
       <c r="G42" s="23"/>
       <c r="H42" s="23"/>
     </row>
-    <row r="43" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="43" spans="2:8" x14ac:dyDescent="0.25">
       <c r="G43" s="23"/>
       <c r="H43" s="23"/>
     </row>
-    <row r="49" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="49" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B49" s="23"/>
       <c r="C49" s="23"/>
       <c r="D49" s="23"/>
@@ -5527,32 +5527,32 @@
       <c r="G49" s="23"/>
       <c r="H49" s="23"/>
     </row>
-    <row r="50" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="50" spans="2:8" x14ac:dyDescent="0.25">
       <c r="F50" s="23"/>
       <c r="G50" s="23"/>
       <c r="H50" s="23"/>
     </row>
-    <row r="51" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="51" spans="2:8" x14ac:dyDescent="0.25">
       <c r="F51" s="23"/>
       <c r="G51" s="23"/>
       <c r="H51" s="23"/>
     </row>
-    <row r="52" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="52" spans="2:8" x14ac:dyDescent="0.25">
       <c r="F52" s="23"/>
       <c r="G52" s="23"/>
       <c r="H52" s="23"/>
     </row>
-    <row r="53" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="53" spans="2:8" x14ac:dyDescent="0.25">
       <c r="F53" s="23"/>
       <c r="G53" s="23"/>
       <c r="H53" s="23"/>
     </row>
-    <row r="54" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="54" spans="2:8" x14ac:dyDescent="0.25">
       <c r="F54" s="23"/>
       <c r="G54" s="23"/>
       <c r="H54" s="23"/>
     </row>
-    <row r="55" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="55" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B55" s="23"/>
       <c r="C55" s="23"/>
       <c r="D55" s="23"/>
@@ -5561,7 +5561,7 @@
       <c r="G55" s="23"/>
       <c r="H55" s="23"/>
     </row>
-    <row r="56" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="56" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B56" s="23"/>
       <c r="C56" s="23"/>
       <c r="D56" s="23"/>
@@ -5570,7 +5570,7 @@
       <c r="G56" s="23"/>
       <c r="H56" s="23"/>
     </row>
-    <row r="57" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="57" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B57" s="23"/>
       <c r="C57" s="23"/>
       <c r="D57" s="23"/>
@@ -5579,7 +5579,7 @@
       <c r="G57" s="23"/>
       <c r="H57" s="23"/>
     </row>
-    <row r="58" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="58" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B58" s="23"/>
       <c r="C58" s="23"/>
       <c r="D58" s="23"/>
@@ -5598,39 +5598,39 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="B2:T58"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.6640625" customWidth="1"/>
-    <col min="2" max="2" width="20.44140625" customWidth="1"/>
-    <col min="3" max="3" width="16.33203125" customWidth="1"/>
-    <col min="4" max="4" width="20.44140625" customWidth="1"/>
+    <col min="1" max="1" width="14.7109375" customWidth="1"/>
+    <col min="2" max="2" width="20.42578125" customWidth="1"/>
+    <col min="3" max="3" width="16.28515625" customWidth="1"/>
+    <col min="4" max="4" width="20.42578125" customWidth="1"/>
     <col min="5" max="5" width="24" customWidth="1"/>
-    <col min="6" max="6" width="21.109375" customWidth="1"/>
-    <col min="7" max="7" width="29.88671875" customWidth="1"/>
-    <col min="8" max="8" width="24.88671875" customWidth="1"/>
-    <col min="9" max="9" width="21.88671875" customWidth="1"/>
-    <col min="10" max="10" width="21.6640625" customWidth="1"/>
-    <col min="11" max="11" width="16.6640625" customWidth="1"/>
+    <col min="6" max="6" width="21.140625" customWidth="1"/>
+    <col min="7" max="7" width="29.85546875" customWidth="1"/>
+    <col min="8" max="8" width="24.85546875" customWidth="1"/>
+    <col min="9" max="9" width="21.85546875" customWidth="1"/>
+    <col min="10" max="10" width="21.7109375" customWidth="1"/>
+    <col min="11" max="11" width="16.7109375" customWidth="1"/>
     <col min="12" max="12" width="26" customWidth="1"/>
-    <col min="13" max="13" width="27.6640625" customWidth="1"/>
-    <col min="14" max="14" width="30.88671875" customWidth="1"/>
-    <col min="15" max="17" width="22.6640625" customWidth="1"/>
-    <col min="18" max="18" width="26.33203125" customWidth="1"/>
-    <col min="19" max="19" width="35.109375" customWidth="1"/>
-    <col min="20" max="20" width="21.5546875" customWidth="1"/>
-    <col min="21" max="22" width="12.6640625" customWidth="1"/>
+    <col min="13" max="13" width="27.7109375" customWidth="1"/>
+    <col min="14" max="14" width="30.85546875" customWidth="1"/>
+    <col min="15" max="17" width="22.7109375" customWidth="1"/>
+    <col min="18" max="18" width="26.28515625" customWidth="1"/>
+    <col min="19" max="19" width="35.140625" customWidth="1"/>
+    <col min="20" max="20" width="21.5703125" customWidth="1"/>
+    <col min="21" max="22" width="12.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:20" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
         <v>188</v>
       </c>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
-      <c r="J2" s="64"/>
-      <c r="K2" s="64"/>
-    </row>
-    <row r="3" spans="2:20" s="23" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="J2" s="65"/>
+      <c r="K2" s="65"/>
+    </row>
+    <row r="3" spans="2:20" s="23" customFormat="1" x14ac:dyDescent="0.25">
       <c r="D3" s="23" t="s">
         <v>206</v>
       </c>
@@ -5640,62 +5640,62 @@
         <v>287</v>
       </c>
     </row>
-    <row r="4" spans="2:20" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="69" t="s">
+    <row r="4" spans="2:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B4" s="62" t="s">
         <v>189</v>
       </c>
-      <c r="C4" s="69" t="s">
+      <c r="C4" s="62" t="s">
         <v>196</v>
       </c>
-      <c r="D4" s="69" t="s">
+      <c r="D4" s="62" t="s">
         <v>205</v>
       </c>
-      <c r="E4" s="69" t="s">
+      <c r="E4" s="62" t="s">
         <v>214</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="F4" s="62" t="s">
         <v>221</v>
       </c>
-      <c r="G4" s="1" t="s">
+      <c r="G4" s="62" t="s">
         <v>229</v>
       </c>
-      <c r="H4" s="1" t="s">
+      <c r="H4" s="62" t="s">
         <v>236</v>
       </c>
-      <c r="I4" s="69" t="s">
+      <c r="I4" s="62" t="s">
         <v>266</v>
       </c>
       <c r="J4" s="1"/>
-      <c r="K4" s="69" t="s">
+      <c r="K4" s="62" t="s">
         <v>244</v>
       </c>
-      <c r="L4" s="1" t="s">
+      <c r="L4" s="62" t="s">
         <v>247</v>
       </c>
       <c r="M4" s="1" t="s">
         <v>250</v>
       </c>
-      <c r="N4" s="1" t="s">
+      <c r="N4" s="62" t="s">
         <v>261</v>
       </c>
       <c r="O4" s="1"/>
-      <c r="P4" s="1" t="s">
+      <c r="P4" s="62" t="s">
         <v>273</v>
       </c>
-      <c r="Q4" s="1" t="s">
+      <c r="Q4" s="62" t="s">
         <v>306</v>
       </c>
-      <c r="R4" s="69" t="s">
+      <c r="R4" s="62" t="s">
         <v>288</v>
       </c>
-      <c r="S4" s="69" t="s">
+      <c r="S4" s="62" t="s">
         <v>297</v>
       </c>
-      <c r="T4" s="69" t="s">
+      <c r="T4" s="62" t="s">
         <v>283</v>
       </c>
     </row>
-    <row r="5" spans="2:20" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="36" t="s">
         <v>190</v>
       </c>
@@ -5750,7 +5750,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="6" spans="2:20" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="2" t="s">
         <v>191</v>
       </c>
@@ -5805,7 +5805,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="7" spans="2:20" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="38" t="s">
         <v>217</v>
       </c>
@@ -5852,7 +5852,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="8" spans="2:20" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="2" t="s">
         <v>417</v>
       </c>
@@ -5891,7 +5891,7 @@
       </c>
       <c r="T8" s="2"/>
     </row>
-    <row r="9" spans="2:20" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="38"/>
       <c r="C9" s="34"/>
       <c r="D9" s="2" t="s">
@@ -5922,7 +5922,7 @@
       </c>
       <c r="T9" s="2"/>
     </row>
-    <row r="10" spans="2:20" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="28"/>
       <c r="C10" s="34"/>
       <c r="D10" s="2" t="s">
@@ -5951,7 +5951,7 @@
       <c r="S10" s="2"/>
       <c r="T10" s="2"/>
     </row>
-    <row r="11" spans="2:20" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="28"/>
       <c r="C11" s="34"/>
       <c r="D11" s="2"/>
@@ -5978,7 +5978,7 @@
       <c r="S11" s="38"/>
       <c r="T11" s="38"/>
     </row>
-    <row r="12" spans="2:20" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="34"/>
       <c r="C12" s="34"/>
       <c r="D12" s="2"/>
@@ -6005,7 +6005,7 @@
       <c r="S12" s="38"/>
       <c r="T12" s="38"/>
     </row>
-    <row r="13" spans="2:20" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B13" s="34"/>
       <c r="C13" s="34"/>
       <c r="D13" s="2"/>
@@ -6029,7 +6029,7 @@
       <c r="S13" s="2"/>
       <c r="T13" s="2"/>
     </row>
-    <row r="14" spans="2:20" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="34"/>
       <c r="C14" s="34"/>
       <c r="D14" s="2"/>
@@ -6054,7 +6054,7 @@
       <c r="S14" s="2"/>
       <c r="T14" s="2"/>
     </row>
-    <row r="15" spans="2:20" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="34"/>
       <c r="C15" s="34"/>
       <c r="D15" s="2"/>
@@ -6075,7 +6075,7 @@
       <c r="S15" s="2"/>
       <c r="T15" s="2"/>
     </row>
-    <row r="16" spans="2:20" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B16" s="34"/>
       <c r="C16" s="34"/>
       <c r="D16" s="2"/>
@@ -6096,7 +6096,7 @@
       <c r="S16" s="2"/>
       <c r="T16" s="2"/>
     </row>
-    <row r="17" spans="2:20" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B17" s="34"/>
       <c r="C17" s="34"/>
       <c r="D17" s="2"/>
@@ -6117,7 +6117,7 @@
       <c r="S17" s="2"/>
       <c r="T17" s="2"/>
     </row>
-    <row r="18" spans="2:20" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B18" s="34"/>
       <c r="C18" s="34"/>
       <c r="D18" s="2"/>
@@ -6138,7 +6138,7 @@
       <c r="S18" s="2"/>
       <c r="T18" s="2"/>
     </row>
-    <row r="19" spans="2:20" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B19" s="34"/>
       <c r="C19" s="34"/>
       <c r="D19" s="2"/>
@@ -6159,7 +6159,7 @@
       <c r="S19" s="2"/>
       <c r="T19" s="2"/>
     </row>
-    <row r="20" spans="2:20" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B20" s="34"/>
       <c r="C20" s="34"/>
       <c r="D20" s="2"/>
@@ -6180,27 +6180,27 @@
       <c r="S20" s="2"/>
       <c r="T20" s="2"/>
     </row>
-    <row r="21" spans="2:20" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:20" x14ac:dyDescent="0.25">
       <c r="I21" t="s">
         <v>207</v>
       </c>
     </row>
-    <row r="22" spans="2:20" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:20" x14ac:dyDescent="0.25">
       <c r="I22" t="s">
         <v>208</v>
       </c>
     </row>
-    <row r="23" spans="2:20" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:20" x14ac:dyDescent="0.25">
       <c r="I23" t="s">
         <v>211</v>
       </c>
     </row>
-    <row r="24" spans="2:20" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:20" x14ac:dyDescent="0.25">
       <c r="I24" t="s">
         <v>210</v>
       </c>
     </row>
-    <row r="25" spans="2:20" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B25" t="s">
         <v>184</v>
       </c>
@@ -6210,15 +6210,15 @@
       <c r="I25" s="15" t="s">
         <v>196</v>
       </c>
-      <c r="J25" s="63" t="s">
+      <c r="J25" s="64" t="s">
         <v>209</v>
       </c>
-      <c r="K25" s="63"/>
+      <c r="K25" s="64"/>
       <c r="N25" t="s">
         <v>278</v>
       </c>
     </row>
-    <row r="26" spans="2:20" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B26" t="s">
         <v>185</v>
       </c>
@@ -6241,7 +6241,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="27" spans="2:20" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B27" t="s">
         <v>186</v>
       </c>
@@ -6265,7 +6265,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="28" spans="2:20" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B28" t="s">
         <v>192</v>
       </c>
@@ -6286,7 +6286,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="2:20" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B29" s="16" t="s">
         <v>187</v>
       </c>
@@ -6303,7 +6303,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="2:20" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:20" x14ac:dyDescent="0.25">
       <c r="F30" t="s">
         <v>221</v>
       </c>
@@ -6320,7 +6320,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="2:20" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:20" x14ac:dyDescent="0.25">
       <c r="F31" s="15" t="s">
         <v>222</v>
       </c>
@@ -6340,7 +6340,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="2:20" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:20" x14ac:dyDescent="0.25">
       <c r="F32" s="15">
         <v>1</v>
       </c>
@@ -6363,7 +6363,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="33" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B33" s="40" t="s">
         <v>250</v>
       </c>
@@ -6389,7 +6389,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B34" s="40" t="s">
         <v>251</v>
       </c>
@@ -6421,7 +6421,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B35" s="43">
         <v>1</v>
       </c>
@@ -6453,7 +6453,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B36" s="43">
         <v>1</v>
       </c>
@@ -6476,7 +6476,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B37" s="43">
         <v>1</v>
       </c>
@@ -6495,7 +6495,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B38" s="43">
         <v>2</v>
       </c>
@@ -6512,7 +6512,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="39" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B39" s="43">
         <v>2</v>
       </c>
@@ -6541,7 +6541,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="40" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B40" s="43">
         <v>2</v>
       </c>
@@ -6568,7 +6568,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="41" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="41" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B41" s="43">
         <v>2</v>
       </c>
@@ -6595,7 +6595,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="42" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="42" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B42" s="43"/>
       <c r="C42" s="43"/>
       <c r="D42" s="43"/>
@@ -6614,7 +6614,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="43" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="43" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B43" s="44"/>
       <c r="C43" s="44"/>
       <c r="D43" s="44"/>
@@ -6631,7 +6631,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="44" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="44" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B44" s="42"/>
       <c r="C44" s="42"/>
       <c r="D44" s="42"/>
@@ -6648,7 +6648,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="45" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="45" spans="2:11" x14ac:dyDescent="0.25">
       <c r="F45" s="15">
         <v>2</v>
       </c>
@@ -6661,7 +6661,7 @@
         <v>666</v>
       </c>
     </row>
-    <row r="46" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="46" spans="2:11" x14ac:dyDescent="0.25">
       <c r="F46" s="15">
         <v>2</v>
       </c>
@@ -6674,7 +6674,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="47" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="47" spans="2:11" x14ac:dyDescent="0.25">
       <c r="F47" s="15">
         <v>2</v>
       </c>
@@ -6687,42 +6687,42 @@
         <v>8</v>
       </c>
     </row>
-    <row r="49" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="49" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E49" t="s">
         <v>298</v>
       </c>
     </row>
-    <row r="50" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="50" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E50" t="s">
         <v>299</v>
       </c>
     </row>
-    <row r="51" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="51" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E51" t="s">
         <v>300</v>
       </c>
     </row>
-    <row r="53" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="53" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E53" t="s">
         <v>301</v>
       </c>
     </row>
-    <row r="54" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="54" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E54" t="s">
         <v>302</v>
       </c>
     </row>
-    <row r="56" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="56" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E56" t="s">
         <v>303</v>
       </c>
     </row>
-    <row r="57" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="57" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E57" t="s">
         <v>304</v>
       </c>
     </row>
-    <row r="58" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="58" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E58" t="s">
         <v>305</v>
       </c>
@@ -6748,19 +6748,19 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{63E46F37-4B03-4545-ABD0-F1F3CE57095A}">
   <dimension ref="A3:L201"/>
-  <sheetFormatPr defaultColWidth="30.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="30.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="10" max="10" width="37.44140625" customWidth="1"/>
-    <col min="11" max="11" width="34.88671875" customWidth="1"/>
+    <col min="10" max="10" width="37.42578125" customWidth="1"/>
+    <col min="11" max="11" width="34.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B3" s="47" t="s">
         <v>418</v>
       </c>
       <c r="C3" s="23"/>
     </row>
-    <row r="4" spans="2:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B4" s="48" t="s">
         <v>419</v>
       </c>
@@ -6774,7 +6774,7 @@
       <c r="I4" s="23"/>
       <c r="J4" s="23"/>
     </row>
-    <row r="5" spans="2:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B5" s="21">
         <v>1</v>
       </c>
@@ -6794,7 +6794,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="6" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B6" s="21">
         <v>2</v>
       </c>
@@ -6814,7 +6814,7 @@
         <v>330</v>
       </c>
     </row>
-    <row r="7" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B7" s="21">
         <v>3</v>
       </c>
@@ -6834,7 +6834,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="8" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B8" s="21">
         <v>4</v>
       </c>
@@ -6854,7 +6854,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="9" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B9" s="21">
         <v>5</v>
       </c>
@@ -6874,7 +6874,7 @@
         <v>339</v>
       </c>
     </row>
-    <row r="10" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B10" s="21">
         <v>6</v>
       </c>
@@ -6894,7 +6894,7 @@
         <v>341</v>
       </c>
     </row>
-    <row r="11" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B11" s="21">
         <v>7</v>
       </c>
@@ -6914,7 +6914,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="12" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:10" x14ac:dyDescent="0.25">
       <c r="G12" s="21">
         <v>7</v>
       </c>
@@ -6928,7 +6928,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="13" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:10" x14ac:dyDescent="0.25">
       <c r="G13" s="21">
         <v>8</v>
       </c>
@@ -6942,7 +6942,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="14" spans="2:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B14" s="47" t="s">
         <v>189</v>
       </c>
@@ -6962,7 +6962,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="15" spans="2:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B15" s="48" t="s">
         <v>190</v>
       </c>
@@ -6988,7 +6988,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="16" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B16" s="21">
         <v>1</v>
       </c>
@@ -7000,7 +7000,7 @@
       </c>
       <c r="E16" s="21"/>
     </row>
-    <row r="17" spans="2:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B17" s="21">
         <v>2</v>
       </c>
@@ -7018,7 +7018,7 @@
       </c>
       <c r="H17" s="23"/>
     </row>
-    <row r="18" spans="2:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B18" s="21">
         <v>3</v>
       </c>
@@ -7041,7 +7041,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="19" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B19" s="21">
         <v>4</v>
       </c>
@@ -7052,13 +7052,13 @@
         <v>2</v>
       </c>
       <c r="E19" s="21"/>
-      <c r="G19" s="68" t="s">
+      <c r="G19" s="69" t="s">
         <v>423</v>
       </c>
-      <c r="H19" s="68"/>
-      <c r="I19" s="68"/>
-    </row>
-    <row r="20" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="H19" s="69"/>
+      <c r="I19" s="69"/>
+    </row>
+    <row r="20" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B20" s="21">
         <v>5</v>
       </c>
@@ -7069,11 +7069,11 @@
         <v>2</v>
       </c>
       <c r="E20" s="21"/>
-      <c r="G20" s="66"/>
-      <c r="H20" s="66"/>
-      <c r="I20" s="66"/>
-    </row>
-    <row r="21" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="G20" s="67"/>
+      <c r="H20" s="67"/>
+      <c r="I20" s="67"/>
+    </row>
+    <row r="21" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B21" s="21">
         <v>6</v>
       </c>
@@ -7084,11 +7084,11 @@
         <v>3</v>
       </c>
       <c r="E21" s="21"/>
-      <c r="G21" s="66"/>
-      <c r="H21" s="66"/>
-      <c r="I21" s="66"/>
-    </row>
-    <row r="22" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="G21" s="67"/>
+      <c r="H21" s="67"/>
+      <c r="I21" s="67"/>
+    </row>
+    <row r="22" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B22" s="21">
         <v>7</v>
       </c>
@@ -7099,11 +7099,11 @@
         <v>3</v>
       </c>
       <c r="E22" s="21"/>
-      <c r="G22" s="66"/>
-      <c r="H22" s="66"/>
-      <c r="I22" s="66"/>
-    </row>
-    <row r="23" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="G22" s="67"/>
+      <c r="H22" s="67"/>
+      <c r="I22" s="67"/>
+    </row>
+    <row r="23" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B23" s="21">
         <v>8</v>
       </c>
@@ -7115,7 +7115,7 @@
       </c>
       <c r="E23" s="21"/>
     </row>
-    <row r="24" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B24" s="21">
         <v>9</v>
       </c>
@@ -7127,7 +7127,7 @@
       </c>
       <c r="E24" s="21"/>
     </row>
-    <row r="25" spans="2:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B25" s="21">
         <v>10</v>
       </c>
@@ -7149,7 +7149,7 @@
       <c r="K25" s="23"/>
       <c r="L25" s="23"/>
     </row>
-    <row r="26" spans="2:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B26" s="21">
         <v>11</v>
       </c>
@@ -7179,7 +7179,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="27" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B27" s="21">
         <v>12</v>
       </c>
@@ -7199,7 +7199,7 @@
       <c r="K27" s="23"/>
       <c r="L27" s="23"/>
     </row>
-    <row r="28" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B28" s="21">
         <v>13</v>
       </c>
@@ -7211,15 +7211,15 @@
       </c>
       <c r="E28" s="21"/>
       <c r="G28" s="23"/>
-      <c r="H28" s="66" t="s">
+      <c r="H28" s="67" t="s">
         <v>421</v>
       </c>
-      <c r="I28" s="66"/>
-      <c r="J28" s="66"/>
-      <c r="K28" s="66"/>
+      <c r="I28" s="67"/>
+      <c r="J28" s="67"/>
+      <c r="K28" s="67"/>
       <c r="L28" s="23"/>
     </row>
-    <row r="29" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B29" s="21">
         <v>14</v>
       </c>
@@ -7231,13 +7231,13 @@
       </c>
       <c r="E29" s="21"/>
       <c r="G29" s="23"/>
-      <c r="H29" s="66"/>
-      <c r="I29" s="66"/>
-      <c r="J29" s="66"/>
-      <c r="K29" s="66"/>
+      <c r="H29" s="67"/>
+      <c r="I29" s="67"/>
+      <c r="J29" s="67"/>
+      <c r="K29" s="67"/>
       <c r="L29" s="23"/>
     </row>
-    <row r="30" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B30" s="21">
         <v>15</v>
       </c>
@@ -7249,13 +7249,13 @@
       </c>
       <c r="E30" s="21"/>
       <c r="G30" s="23"/>
-      <c r="H30" s="66"/>
-      <c r="I30" s="66"/>
-      <c r="J30" s="66"/>
-      <c r="K30" s="66"/>
+      <c r="H30" s="67"/>
+      <c r="I30" s="67"/>
+      <c r="J30" s="67"/>
+      <c r="K30" s="67"/>
       <c r="L30" s="23"/>
     </row>
-    <row r="31" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B31" s="21">
         <v>16</v>
       </c>
@@ -7267,13 +7267,13 @@
       </c>
       <c r="E31" s="21"/>
       <c r="G31" s="23"/>
-      <c r="H31" s="66"/>
-      <c r="I31" s="66"/>
-      <c r="J31" s="66"/>
-      <c r="K31" s="66"/>
+      <c r="H31" s="67"/>
+      <c r="I31" s="67"/>
+      <c r="J31" s="67"/>
+      <c r="K31" s="67"/>
       <c r="L31" s="23"/>
     </row>
-    <row r="32" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B32" s="21">
         <v>17</v>
       </c>
@@ -7284,12 +7284,12 @@
         <v>6</v>
       </c>
       <c r="E32" s="21"/>
-      <c r="H32" s="66"/>
-      <c r="I32" s="66"/>
-      <c r="J32" s="66"/>
-      <c r="K32" s="66"/>
-    </row>
-    <row r="33" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="H32" s="67"/>
+      <c r="I32" s="67"/>
+      <c r="J32" s="67"/>
+      <c r="K32" s="67"/>
+    </row>
+    <row r="33" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B33" s="21">
         <v>18</v>
       </c>
@@ -7300,12 +7300,12 @@
         <v>5</v>
       </c>
       <c r="E33" s="21"/>
-      <c r="H33" s="66"/>
-      <c r="I33" s="66"/>
-      <c r="J33" s="66"/>
-      <c r="K33" s="66"/>
-    </row>
-    <row r="34" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="H33" s="67"/>
+      <c r="I33" s="67"/>
+      <c r="J33" s="67"/>
+      <c r="K33" s="67"/>
+    </row>
+    <row r="34" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B34" s="21">
         <v>19</v>
       </c>
@@ -7316,12 +7316,12 @@
         <v>7</v>
       </c>
       <c r="E34" s="21"/>
-      <c r="H34" s="66"/>
-      <c r="I34" s="66"/>
-      <c r="J34" s="66"/>
-      <c r="K34" s="66"/>
-    </row>
-    <row r="35" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="H34" s="67"/>
+      <c r="I34" s="67"/>
+      <c r="J34" s="67"/>
+      <c r="K34" s="67"/>
+    </row>
+    <row r="35" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B35" s="21">
         <v>20</v>
       </c>
@@ -7335,17 +7335,17 @@
         <v>19</v>
       </c>
     </row>
-    <row r="37" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:11" x14ac:dyDescent="0.25">
       <c r="D37" s="54" t="s">
         <v>427</v>
       </c>
     </row>
-    <row r="38" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:11" x14ac:dyDescent="0.25">
       <c r="D38" t="s">
         <v>428</v>
       </c>
     </row>
-    <row r="39" spans="2:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:11" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B39" s="47" t="s">
         <v>244</v>
       </c>
@@ -7353,7 +7353,7 @@
         <v>429</v>
       </c>
     </row>
-    <row r="40" spans="2:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:11" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B40" s="48" t="s">
         <v>245</v>
       </c>
@@ -7361,7 +7361,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="41" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B41" s="21">
         <v>1</v>
       </c>
@@ -7369,7 +7369,7 @@
         <v>432</v>
       </c>
     </row>
-    <row r="42" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="42" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B42" s="21">
         <v>2</v>
       </c>
@@ -7377,7 +7377,7 @@
         <v>430</v>
       </c>
     </row>
-    <row r="43" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="43" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B43" s="21">
         <v>3</v>
       </c>
@@ -7385,7 +7385,7 @@
         <v>431</v>
       </c>
     </row>
-    <row r="44" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="44" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B44" s="21">
         <v>4</v>
       </c>
@@ -7393,7 +7393,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="45" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="45" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B45" s="21">
         <v>5</v>
       </c>
@@ -7401,7 +7401,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="46" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="46" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B46" s="21">
         <v>6</v>
       </c>
@@ -7409,7 +7409,7 @@
         <v>435</v>
       </c>
     </row>
-    <row r="47" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="47" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B47" s="21">
         <v>7</v>
       </c>
@@ -7417,7 +7417,7 @@
         <v>479</v>
       </c>
     </row>
-    <row r="48" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="48" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B48" s="21">
         <v>8</v>
       </c>
@@ -7425,12 +7425,12 @@
         <v>316</v>
       </c>
     </row>
-    <row r="51" spans="2:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="51" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B51" s="47" t="s">
         <v>236</v>
       </c>
     </row>
-    <row r="52" spans="2:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="52" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B52" s="48" t="s">
         <v>237</v>
       </c>
@@ -7455,15 +7455,15 @@
       <c r="I52" s="2" t="s">
         <v>424</v>
       </c>
-      <c r="J52" s="67" t="s">
+      <c r="J52" s="68" t="s">
         <v>425</v>
       </c>
-      <c r="K52" s="67"/>
+      <c r="K52" s="68"/>
       <c r="L52" s="2" t="s">
         <v>426</v>
       </c>
     </row>
-    <row r="53" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="53" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B53" s="21">
         <v>1</v>
       </c>
@@ -7492,7 +7492,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="54" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="54" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B54" s="21">
         <v>2</v>
       </c>
@@ -7523,7 +7523,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="55" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="55" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B55" s="21">
         <v>3</v>
       </c>
@@ -7554,7 +7554,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="56" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="56" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B56" s="21">
         <v>4</v>
       </c>
@@ -7585,7 +7585,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="57" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="57" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B57" s="21">
         <v>5</v>
       </c>
@@ -7616,7 +7616,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="58" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="58" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B58" s="21">
         <v>6</v>
       </c>
@@ -7645,7 +7645,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="59" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="59" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B59" s="21">
         <v>7</v>
       </c>
@@ -7674,7 +7674,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="60" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="60" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B60" s="21">
         <v>8</v>
       </c>
@@ -7703,7 +7703,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="61" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="61" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B61" s="21">
         <v>9</v>
       </c>
@@ -7732,7 +7732,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="62" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="62" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B62" s="21">
         <v>10</v>
       </c>
@@ -7761,15 +7761,15 @@
         <v>1</v>
       </c>
     </row>
-    <row r="63" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="63" spans="2:12" x14ac:dyDescent="0.25">
       <c r="L63" s="4"/>
     </row>
-    <row r="65" spans="2:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="65" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B65" s="47" t="s">
         <v>266</v>
       </c>
     </row>
-    <row r="66" spans="2:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="66" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B66" s="48" t="s">
         <v>267</v>
       </c>
@@ -7791,10 +7791,10 @@
       <c r="H66" s="2" t="s">
         <v>451</v>
       </c>
-      <c r="I66" s="67" t="s">
+      <c r="I66" s="68" t="s">
         <v>452</v>
       </c>
-      <c r="J66" s="67"/>
+      <c r="J66" s="68"/>
       <c r="K66" s="2" t="s">
         <v>453</v>
       </c>
@@ -7802,7 +7802,7 @@
         <v>454</v>
       </c>
     </row>
-    <row r="67" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="67" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B67" s="21">
         <v>1</v>
       </c>
@@ -7831,7 +7831,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="68" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="68" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B68" s="21">
         <v>2</v>
       </c>
@@ -7862,7 +7862,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="69" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="69" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B69" s="21">
         <v>3</v>
       </c>
@@ -7893,7 +7893,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="70" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="70" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B70" s="21">
         <v>4</v>
       </c>
@@ -7924,7 +7924,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="71" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="71" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B71" s="21">
         <v>5</v>
       </c>
@@ -7955,7 +7955,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="72" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="72" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B72" s="21">
         <v>6</v>
       </c>
@@ -7984,7 +7984,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="73" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="73" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B73" s="21">
         <v>7</v>
       </c>
@@ -8013,7 +8013,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="74" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="74" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B74" s="21">
         <v>8</v>
       </c>
@@ -8042,7 +8042,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="75" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="75" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B75" s="21">
         <v>9</v>
       </c>
@@ -8071,7 +8071,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="76" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="76" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B76" s="21">
         <v>10</v>
       </c>
@@ -8100,7 +8100,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="77" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="77" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B77" s="21">
         <v>11</v>
       </c>
@@ -8129,7 +8129,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="78" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="78" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B78" s="21">
         <v>12</v>
       </c>
@@ -8158,7 +8158,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="79" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="79" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B79" s="21">
         <v>13</v>
       </c>
@@ -8187,13 +8187,13 @@
         <v>8</v>
       </c>
     </row>
-    <row r="82" spans="2:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="82" spans="2:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B82" s="47" t="s">
         <v>261</v>
       </c>
       <c r="C82" s="23"/>
     </row>
-    <row r="83" spans="2:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="83" spans="2:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B83" s="48" t="s">
         <v>461</v>
       </c>
@@ -8201,7 +8201,7 @@
         <v>462</v>
       </c>
     </row>
-    <row r="84" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="84" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B84" s="21">
         <v>1</v>
       </c>
@@ -8209,7 +8209,7 @@
         <v>329</v>
       </c>
     </row>
-    <row r="85" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="85" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B85" s="21">
         <v>2</v>
       </c>
@@ -8217,7 +8217,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="86" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="86" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B86" s="21">
         <v>3</v>
       </c>
@@ -8225,7 +8225,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="87" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="87" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B87" s="21">
         <v>4</v>
       </c>
@@ -8233,15 +8233,15 @@
         <v>338</v>
       </c>
     </row>
-    <row r="88" spans="2:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="88" spans="2:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B88" s="49"/>
     </row>
-    <row r="89" spans="2:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="89" spans="2:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B89" s="47" t="s">
         <v>229</v>
       </c>
     </row>
-    <row r="90" spans="2:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="90" spans="2:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B90" s="48" t="s">
         <v>230</v>
       </c>
@@ -8267,7 +8267,7 @@
         <v>416</v>
       </c>
     </row>
-    <row r="91" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="91" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B91" s="21">
         <v>1</v>
       </c>
@@ -8293,7 +8293,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="92" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="92" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B92" s="21">
         <v>2</v>
       </c>
@@ -8319,7 +8319,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="93" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="93" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B93" s="21">
         <v>3</v>
       </c>
@@ -8345,7 +8345,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="94" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="94" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B94" s="21">
         <v>4</v>
       </c>
@@ -8371,7 +8371,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="95" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="95" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B95" s="21">
         <v>5</v>
       </c>
@@ -8397,7 +8397,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="96" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="96" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B96" s="21">
         <v>6</v>
       </c>
@@ -8423,7 +8423,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="97" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B97" s="21">
         <v>7</v>
       </c>
@@ -8449,7 +8449,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="98" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B98" s="21">
         <v>8</v>
       </c>
@@ -8475,7 +8475,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="99" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B99" s="21">
         <v>9</v>
       </c>
@@ -8501,7 +8501,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="100" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B100" s="21">
         <v>10</v>
       </c>
@@ -8527,7 +8527,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="101" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A101" s="23" t="s">
         <v>477</v>
       </c>
@@ -8556,7 +8556,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="102" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A102" s="23" t="s">
         <v>477</v>
       </c>
@@ -8585,7 +8585,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="103" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A103" s="23" t="s">
         <v>477</v>
       </c>
@@ -8614,12 +8614,12 @@
         <v>6</v>
       </c>
     </row>
-    <row r="107" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B107" s="47" t="s">
         <v>273</v>
       </c>
     </row>
-    <row r="108" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B108" s="48" t="s">
         <v>274</v>
       </c>
@@ -8633,62 +8633,62 @@
         <v>277</v>
       </c>
     </row>
-    <row r="110" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="B110" s="66" t="s">
+    <row r="110" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B110" s="67" t="s">
         <v>476</v>
       </c>
-      <c r="C110" s="64"/>
-      <c r="D110" s="64"/>
-      <c r="E110" s="64"/>
-    </row>
-    <row r="111" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="B111" s="64"/>
-      <c r="C111" s="64"/>
-      <c r="D111" s="64"/>
-      <c r="E111" s="64"/>
-    </row>
-    <row r="112" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="B112" s="64"/>
-      <c r="C112" s="64"/>
-      <c r="D112" s="64"/>
-      <c r="E112" s="64"/>
-    </row>
-    <row r="113" spans="2:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B113" s="64"/>
-      <c r="C113" s="64"/>
-      <c r="D113" s="64"/>
-      <c r="E113" s="64"/>
+      <c r="C110" s="65"/>
+      <c r="D110" s="65"/>
+      <c r="E110" s="65"/>
+    </row>
+    <row r="111" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B111" s="65"/>
+      <c r="C111" s="65"/>
+      <c r="D111" s="65"/>
+      <c r="E111" s="65"/>
+    </row>
+    <row r="112" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B112" s="65"/>
+      <c r="C112" s="65"/>
+      <c r="D112" s="65"/>
+      <c r="E112" s="65"/>
+    </row>
+    <row r="113" spans="2:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B113" s="65"/>
+      <c r="C113" s="65"/>
+      <c r="D113" s="65"/>
+      <c r="E113" s="65"/>
       <c r="F113" s="23"/>
       <c r="G113" s="23"/>
       <c r="H113" s="23"/>
       <c r="I113" s="23"/>
     </row>
-    <row r="114" spans="2:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B114" s="64"/>
-      <c r="C114" s="64"/>
-      <c r="D114" s="64"/>
-      <c r="E114" s="64"/>
+    <row r="114" spans="2:9" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B114" s="65"/>
+      <c r="C114" s="65"/>
+      <c r="D114" s="65"/>
+      <c r="E114" s="65"/>
       <c r="F114" s="58"/>
       <c r="G114" s="58"/>
       <c r="H114" s="59"/>
       <c r="I114" s="59"/>
     </row>
-    <row r="115" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B115" s="64"/>
-      <c r="C115" s="64"/>
-      <c r="D115" s="64"/>
-      <c r="E115" s="64"/>
+    <row r="115" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B115" s="65"/>
+      <c r="C115" s="65"/>
+      <c r="D115" s="65"/>
+      <c r="E115" s="65"/>
       <c r="G115" s="23"/>
     </row>
-    <row r="116" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="116" spans="2:9" x14ac:dyDescent="0.25">
       <c r="D116" s="23"/>
       <c r="G116" s="23"/>
     </row>
-    <row r="117" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="117" spans="2:9" x14ac:dyDescent="0.25">
       <c r="D117" s="23"/>
       <c r="G117" s="23"/>
     </row>
-    <row r="118" spans="2:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="118" spans="2:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B118" s="47" t="s">
         <v>306</v>
       </c>
@@ -8696,7 +8696,7 @@
       <c r="D118" s="23"/>
       <c r="G118" s="23"/>
     </row>
-    <row r="119" spans="2:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="119" spans="2:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B119" s="48" t="s">
         <v>279</v>
       </c>
@@ -8708,27 +8708,27 @@
       </c>
       <c r="G119" s="23"/>
     </row>
-    <row r="120" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B120" s="65" t="s">
+    <row r="120" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B120" s="66" t="s">
         <v>415</v>
       </c>
-      <c r="C120" s="65"/>
-      <c r="D120" s="65"/>
+      <c r="C120" s="66"/>
+      <c r="D120" s="66"/>
       <c r="G120" s="23"/>
     </row>
-    <row r="121" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B121" s="65"/>
-      <c r="C121" s="65"/>
-      <c r="D121" s="65"/>
+    <row r="121" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B121" s="66"/>
+      <c r="C121" s="66"/>
+      <c r="D121" s="66"/>
       <c r="G121" s="23"/>
     </row>
-    <row r="122" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B122" s="65"/>
-      <c r="C122" s="65"/>
-      <c r="D122" s="65"/>
+    <row r="122" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B122" s="66"/>
+      <c r="C122" s="66"/>
+      <c r="D122" s="66"/>
       <c r="G122" s="23"/>
     </row>
-    <row r="123" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="123" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B123" s="21">
         <v>1</v>
       </c>
@@ -8740,7 +8740,7 @@
       </c>
       <c r="G123" s="23"/>
     </row>
-    <row r="124" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="124" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B124" s="21">
         <v>1</v>
       </c>
@@ -8752,7 +8752,7 @@
       </c>
       <c r="G124" s="23"/>
     </row>
-    <row r="125" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="125" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B125" s="21">
         <v>2</v>
       </c>
@@ -8764,7 +8764,7 @@
       </c>
       <c r="G125" s="23"/>
     </row>
-    <row r="126" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="126" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B126" s="21">
         <v>2</v>
       </c>
@@ -8776,7 +8776,7 @@
       </c>
       <c r="G126" s="23"/>
     </row>
-    <row r="127" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="127" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B127" s="21">
         <v>3</v>
       </c>
@@ -8788,7 +8788,7 @@
       </c>
       <c r="G127" s="23"/>
     </row>
-    <row r="128" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="128" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B128" s="21">
         <v>3</v>
       </c>
@@ -8799,7 +8799,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="129" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="129" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B129" s="21">
         <v>4</v>
       </c>
@@ -8810,7 +8810,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="130" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="130" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B130" s="21">
         <v>4</v>
       </c>
@@ -8821,7 +8821,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="131" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="131" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B131" s="21">
         <v>5</v>
       </c>
@@ -8832,7 +8832,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="132" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="132" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B132" s="21">
         <v>5</v>
       </c>
@@ -8843,7 +8843,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="133" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="133" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B133" s="21">
         <v>5</v>
       </c>
@@ -8854,7 +8854,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="134" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="134" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B134" s="21">
         <v>5</v>
       </c>
@@ -8865,7 +8865,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="135" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="135" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B135" s="21">
         <v>6</v>
       </c>
@@ -8876,7 +8876,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="136" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="136" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B136" s="21">
         <v>7</v>
       </c>
@@ -8887,7 +8887,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="137" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="137" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B137" s="21">
         <v>8</v>
       </c>
@@ -8898,7 +8898,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="138" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="138" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B138" s="21">
         <v>8</v>
       </c>
@@ -8909,7 +8909,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="139" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="139" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B139" s="21">
         <v>8</v>
       </c>
@@ -8920,7 +8920,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="140" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="140" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B140" s="21">
         <v>9</v>
       </c>
@@ -8931,7 +8931,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="141" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="141" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B141" s="21">
         <v>9</v>
       </c>
@@ -8942,7 +8942,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="142" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="142" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B142" s="21">
         <v>9</v>
       </c>
@@ -8953,7 +8953,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="143" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="143" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B143" s="21">
         <v>9</v>
       </c>
@@ -8964,7 +8964,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="144" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="144" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B144" s="21">
         <v>9</v>
       </c>
@@ -8975,7 +8975,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="145" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="145" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B145" s="21">
         <v>10</v>
       </c>
@@ -8986,7 +8986,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="146" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="146" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B146" s="21">
         <v>10</v>
       </c>
@@ -8997,7 +8997,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="147" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="147" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B147" s="21">
         <v>11</v>
       </c>
@@ -9008,7 +9008,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="148" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="148" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B148" s="21">
         <v>11</v>
       </c>
@@ -9019,7 +9019,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="149" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="149" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B149" s="21">
         <v>11</v>
       </c>
@@ -9030,7 +9030,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="150" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="150" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B150" s="21">
         <v>11</v>
       </c>
@@ -9041,7 +9041,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="151" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="151" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B151" s="21">
         <v>11</v>
       </c>
@@ -9052,7 +9052,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="152" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="152" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B152" s="21">
         <v>11</v>
       </c>
@@ -9063,7 +9063,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="153" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="153" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B153" s="21">
         <v>12</v>
       </c>
@@ -9074,7 +9074,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="154" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="154" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B154" s="21">
         <v>13</v>
       </c>
@@ -9085,7 +9085,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="155" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="155" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B155" s="21">
         <v>13</v>
       </c>
@@ -9096,12 +9096,12 @@
         <v>2</v>
       </c>
     </row>
-    <row r="159" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="159" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B159" s="1" t="s">
         <v>288</v>
       </c>
     </row>
-    <row r="160" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="160" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B160" s="36" t="s">
         <v>289</v>
       </c>
@@ -9112,35 +9112,35 @@
         <v>291</v>
       </c>
     </row>
-    <row r="161" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="161" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B161" s="21">
         <v>1</v>
       </c>
       <c r="C161" s="21"/>
       <c r="D161" s="21"/>
     </row>
-    <row r="162" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="162" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B162" s="21">
         <v>2</v>
       </c>
       <c r="C162" s="21"/>
       <c r="D162" s="21"/>
     </row>
-    <row r="163" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="163" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B163" s="21">
         <v>3</v>
       </c>
       <c r="C163" s="21"/>
       <c r="D163" s="21"/>
     </row>
-    <row r="164" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="164" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B164" s="21">
         <v>4</v>
       </c>
       <c r="C164" s="21"/>
       <c r="D164" s="21"/>
     </row>
-    <row r="165" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="165" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B165" s="21">
         <v>5</v>
       </c>
@@ -9151,7 +9151,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="166" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="166" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B166" s="21">
         <v>6</v>
       </c>
@@ -9160,40 +9160,40 @@
         <v>480</v>
       </c>
     </row>
-    <row r="167" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="167" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B167" s="21">
         <v>7</v>
       </c>
       <c r="C167" s="21"/>
       <c r="D167" s="21"/>
     </row>
-    <row r="168" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="168" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B168" s="21">
         <v>8</v>
       </c>
       <c r="C168" s="21"/>
       <c r="D168" s="21"/>
     </row>
-    <row r="169" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="169" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B169" s="21">
         <v>9</v>
       </c>
       <c r="C169" s="21"/>
       <c r="D169" s="21"/>
     </row>
-    <row r="170" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="170" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B170" s="21">
         <v>10</v>
       </c>
       <c r="C170" s="21"/>
       <c r="D170" s="21"/>
     </row>
-    <row r="173" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="173" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B173" s="1" t="s">
         <v>283</v>
       </c>
     </row>
-    <row r="174" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="174" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B174" s="30" t="s">
         <v>284</v>
       </c>
@@ -9204,7 +9204,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="175" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="175" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B175" s="3">
         <v>1</v>
       </c>
@@ -9215,7 +9215,7 @@
         <v>12345</v>
       </c>
     </row>
-    <row r="176" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="176" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B176" s="3">
         <v>2</v>
       </c>
@@ -9226,7 +9226,7 @@
         <v>23456</v>
       </c>
     </row>
-    <row r="177" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="177" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B177" s="3">
         <v>3</v>
       </c>
@@ -9237,7 +9237,7 @@
         <v>34567</v>
       </c>
     </row>
-    <row r="178" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="178" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B178" s="3">
         <v>4</v>
       </c>
@@ -9248,7 +9248,7 @@
         <v>72727</v>
       </c>
     </row>
-    <row r="179" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="179" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B179" s="3">
         <v>5</v>
       </c>
@@ -9259,7 +9259,7 @@
         <v>28282</v>
       </c>
     </row>
-    <row r="182" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="182" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B182" s="1" t="s">
         <v>297</v>
       </c>
@@ -9268,7 +9268,7 @@
       <c r="E182" s="23"/>
       <c r="F182" s="23"/>
     </row>
-    <row r="183" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="183" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B183" s="36" t="s">
         <v>293</v>
       </c>
@@ -9285,7 +9285,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="184" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="184" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B184" s="23" t="s">
         <v>487</v>
       </c>
@@ -9302,14 +9302,14 @@
         <v>491</v>
       </c>
     </row>
-    <row r="185" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="185" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B185" s="23"/>
       <c r="C185" s="23"/>
       <c r="D185" s="23"/>
       <c r="E185" s="23"/>
       <c r="F185" s="23"/>
     </row>
-    <row r="186" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="186" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B186" s="23">
         <v>1</v>
       </c>
@@ -9320,7 +9320,7 @@
       <c r="E186" s="23"/>
       <c r="F186" s="23"/>
     </row>
-    <row r="187" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="187" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B187" s="23">
         <v>2</v>
       </c>
@@ -9331,7 +9331,7 @@
       <c r="E187" s="23"/>
       <c r="F187" s="23"/>
     </row>
-    <row r="188" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="188" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B188" s="23">
         <v>3</v>
       </c>
@@ -9342,7 +9342,7 @@
       <c r="E188" s="23"/>
       <c r="F188" s="23"/>
     </row>
-    <row r="189" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="189" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B189" s="23">
         <v>4</v>
       </c>
@@ -9353,7 +9353,7 @@
       <c r="E189" s="23"/>
       <c r="F189" s="23"/>
     </row>
-    <row r="190" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="190" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B190" s="23">
         <v>5</v>
       </c>
@@ -9364,7 +9364,7 @@
       <c r="E190" s="23"/>
       <c r="F190" s="23"/>
     </row>
-    <row r="191" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="191" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B191" s="23">
         <v>6</v>
       </c>
@@ -9375,7 +9375,7 @@
       <c r="E191" s="23"/>
       <c r="F191" s="23"/>
     </row>
-    <row r="192" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="192" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B192" s="23"/>
       <c r="C192" s="23" t="s">
         <v>490</v>
@@ -9384,7 +9384,7 @@
       <c r="E192" s="23"/>
       <c r="F192" s="23"/>
     </row>
-    <row r="193" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="193" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B193" s="23">
         <v>10</v>
       </c>
@@ -9395,7 +9395,7 @@
       <c r="E193" s="23"/>
       <c r="F193" s="23"/>
     </row>
-    <row r="194" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="194" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B194" s="23">
         <v>1</v>
       </c>
@@ -9406,7 +9406,7 @@
       <c r="E194" s="23"/>
       <c r="F194" s="23"/>
     </row>
-    <row r="195" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="195" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B195" s="23"/>
       <c r="C195" s="23" t="s">
         <v>490</v>
@@ -9415,7 +9415,7 @@
       <c r="E195" s="23"/>
       <c r="F195" s="23"/>
     </row>
-    <row r="196" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="196" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B196" s="23">
         <v>10</v>
       </c>
@@ -9426,7 +9426,7 @@
       <c r="E196" s="4"/>
       <c r="F196" s="4"/>
     </row>
-    <row r="197" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="197" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B197" s="4"/>
       <c r="C197" s="4" t="s">
         <v>490</v>
@@ -9435,7 +9435,7 @@
       <c r="E197" s="4"/>
       <c r="F197" s="4"/>
     </row>
-    <row r="198" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="198" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B198" s="61">
         <v>3</v>
       </c>
@@ -9446,7 +9446,7 @@
       <c r="E198" s="4"/>
       <c r="F198" s="4"/>
     </row>
-    <row r="199" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="199" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B199" s="61">
         <v>6</v>
       </c>
@@ -9457,7 +9457,7 @@
       <c r="E199" s="4"/>
       <c r="F199" s="4"/>
     </row>
-    <row r="200" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="200" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B200" s="61">
         <v>9</v>
       </c>
@@ -9468,7 +9468,7 @@
       <c r="E200" s="4"/>
       <c r="F200" s="4"/>
     </row>
-    <row r="201" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="201" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B201" s="4"/>
       <c r="C201" s="4"/>
       <c r="D201" s="4"/>

</xml_diff>

<commit_message>
Finish creating test data - 13.04.2025
</commit_message>
<xml_diff>
--- a/1. Database Design/Java23 QuyenPhan Database Design.xlsx
+++ b/1. Database Design/Java23 QuyenPhan Database Design.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\qphan\Desktop\bkit\course - webapp\java23\3. Database\1. Database Design\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2E68749-AECD-42AF-B262-33C7D66849E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{073230FE-10E8-482F-9BB5-82DDDD166741}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" tabRatio="588" firstSheet="3" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" tabRatio="588" firstSheet="3" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="B1. Mô hình quan niệm" sheetId="1" r:id="rId1"/>
@@ -5672,7 +5672,7 @@
       <c r="L4" s="62" t="s">
         <v>247</v>
       </c>
-      <c r="M4" s="1" t="s">
+      <c r="M4" s="62" t="s">
         <v>250</v>
       </c>
       <c r="N4" s="62" t="s">

</xml_diff>